<commit_message>
Remaining changes to volunteers report
</commit_message>
<xml_diff>
--- a/test/fixtures/files/invalid_volunteer_type.xlsx
+++ b/test/fixtures/files/invalid_volunteer_type.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="19">
   <si>
     <t>RowID</t>
   </si>
@@ -25,6 +25,9 @@
     <t>Name</t>
   </si>
   <si>
+    <t>Department</t>
+  </si>
+  <si>
     <t>SportRelated</t>
   </si>
   <si>
@@ -53,6 +56,9 @@
   </si>
   <si>
     <t>Caffeine Gopher</t>
+  </si>
+  <si>
+    <t>Online</t>
   </si>
   <si>
     <t>FALSE</t>
@@ -82,7 +88,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -114,13 +120,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
@@ -427,22 +436,23 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" style="3" width="8.576428571428572" customWidth="1" bestFit="1"/>
     <col min="2" max="2" style="3" width="6.719285714285714" customWidth="1" bestFit="1"/>
     <col min="3" max="3" style="3" width="14.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="3" width="12.005" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="3" width="6.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="3" width="55.57642857142857" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="3" width="12.005" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="3" width="6.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="3" width="55.57642857142857" customWidth="1" bestFit="1"/>
     <col min="8" max="8" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="3" width="12.005" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="3" width="12.005" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -452,7 +462,7 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
@@ -464,44 +474,50 @@
       <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
       <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="2" t="s">
         <v>9</v>
       </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
       <c r="A2" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="D2" s="1" t="s">
         <v>13</v>
       </c>
+      <c r="D2" s="2" t="s">
+        <v>14</v>
+      </c>
       <c r="E2" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G2" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="I2" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="H2" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="I2" s="2"/>
-      <c r="J2" s="1" t="s">
-        <v>16</v>
+      <c r="J2" s="2"/>
+      <c r="K2" s="1" t="s">
+        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>